<commit_message>
Opdateret HejDoktors testresultet på XDIS'er
</commit_message>
<xml_diff>
--- a/html/Alle systemer (Samlet liste)_excel.XLSX
+++ b/html/Alle systemer (Samlet liste)_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://medcomdk-my.sharepoint.com/personal/sof_medcom_dk/Documents/Dokumenter/GitHub/GodkendteSystemer/html/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_BEA61AB9872538EA9D6B3A0756B6BD6E70CF7E84" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAFF3D9A-8871-4777-93A3-83B73D0B50D4}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_BEA61AB97205BACAD768370756B6BD6E70CF7EB2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{419535D0-8B3F-47C7-8D7A-02598116BD05}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29956,7 +29956,7 @@
         <v>15</v>
       </c>
       <c r="G1210" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1211" spans="1:7" x14ac:dyDescent="0.35">
@@ -30002,7 +30002,7 @@
         <v>15</v>
       </c>
       <c r="G1212" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1213" spans="1:7" x14ac:dyDescent="0.35">
@@ -30025,7 +30025,7 @@
         <v>15</v>
       </c>
       <c r="G1213" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1214" spans="1:7" x14ac:dyDescent="0.35">
@@ -30163,7 +30163,7 @@
         <v>15</v>
       </c>
       <c r="G1219" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1220" spans="1:7" x14ac:dyDescent="0.35">
@@ -30393,7 +30393,7 @@
         <v>15</v>
       </c>
       <c r="G1229" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="1230" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>